<commit_message>
sims: v4 rename book_per_equity -> LP_leverage for clarity (entry 495)
Operator asked where leverage went. It was present as book_per_equity
(+ borrow_APR) — the leverage on the Temporal/options side, HLP un-levered
(entry 486) — but the rename obscured it. Renamed the Assumptions label back
to LP_leverage + explicit note; NOTES updated; formulas unchanged (reference
the cell, not the name). Verified 1x->2x doubles the options edge, HLP flat.
Transcript 495.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cs1cJ4yQMcmxqbEVrDpqHd
</commit_message>
<xml_diff>
--- a/sims/temporal_lp_economics_MODEL_v4_options_seller_CORRECTED.xlsx
+++ b/sims/temporal_lp_economics_MODEL_v4_options_seller_CORRECTED.xlsx
@@ -790,7 +790,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>book_per_equity</t>
+          <t>LP_leverage</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
@@ -798,7 +798,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>option VALUE the LP is short per $ equity (normalization; LOAD-BEARING).</t>
+          <t>LEVERAGE on the Temporal/options side = option value short per $ of equity (1.0x = unlevered). HLP is additive at margin and NOT levered (per entry 486). borrow_APR below is its financing cost.</t>
         </is>
       </c>
     </row>

</xml_diff>